<commit_message>
Render study evidence inline and plan Day 12
</commit_message>
<xml_diff>
--- a/HDLBits_Tracker.xlsx
+++ b/HDLBits_Tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rff753c5e07404c55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2073de9ca2e24fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb227a53ac6834bc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rde6eb7f34cc24e36"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2281,7 +2281,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2353,6 +2353,16 @@
         <x:fgColor rgb="FFCCFFCC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E1F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFF99"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="7">
     <x:border/>
@@ -2415,7 +2425,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="74">
+  <x:cellXfs count="79">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2610,6 +2620,11 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="14" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Hyperlink" xfId="1"/>
@@ -2941,7 +2956,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F5" s="33" t="str">
-        <x:v>Day 11 plan</x:v>
+        <x:v>Day 12 plan</x:v>
       </x:c>
       <x:c r="G5" s="33" t="s">
         <x:v>5</x:v>
@@ -2971,7 +2986,7 @@
         <x:v>Date</x:v>
       </x:c>
       <x:c r="G6" s="62" t="n">
-        <x:v>46207</x:v>
+        <x:v>46208</x:v>
       </x:c>
       <x:c r="H6" s="34"/>
     </x:row>
@@ -2995,7 +3010,7 @@
         <x:v>Queue</x:v>
       </x:c>
       <x:c r="G8" s="63" t="str">
-        <x:v>study/Day 11.md</x:v>
+        <x:v>study/Day 12.md</x:v>
       </x:c>
       <x:c r="H8" s="35"/>
     </x:row>
@@ -3309,6 +3324,15 @@
       </x:c>
     </x:row>
     <x:row r="22">
+      <x:c r="A22" s="75" t="str">
+        <x:v>Day 12</x:v>
+      </x:c>
+      <x:c r="B22" s="71" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="C22" s="78" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="E22" s="25" t="s">
         <x:v>28</x:v>
       </x:c>
@@ -3904,7 +3928,7 @@
       <x:c r="A11" s="3">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B11" s="3">
+      <x:c r="B11" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C11" s="2" t="s">
@@ -3922,8 +3946,8 @@
       <x:c r="G11" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H11" s="3" t="s">
-        <x:v>13</x:v>
+      <x:c r="H11" s="3" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I11" s="56">
         <x:v>46196</x:v>
@@ -3971,7 +3995,7 @@
       <x:c r="A12" s="7">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B12" s="7">
+      <x:c r="B12" s="7" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C12" s="8" t="s">
@@ -3989,8 +4013,8 @@
       <x:c r="G12" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H12" s="7" t="s">
-        <x:v>13</x:v>
+      <x:c r="H12" s="7" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I12" s="55">
         <x:v>46196</x:v>
@@ -4038,7 +4062,7 @@
       <x:c r="A13" s="3">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B13" s="3">
+      <x:c r="B13" s="3" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="C13" s="2" t="s">
@@ -4056,8 +4080,8 @@
       <x:c r="G13" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H13" s="3" t="s">
-        <x:v>13</x:v>
+      <x:c r="H13" s="3" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I13" s="56">
         <x:v>46196</x:v>
@@ -4105,7 +4129,7 @@
       <x:c r="A14" s="7">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B14" s="7">
+      <x:c r="B14" s="7" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C14" s="8" t="s">
@@ -4123,8 +4147,8 @@
       <x:c r="G14" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H14" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H14" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I14" s="55">
         <x:v>46197</x:v>
@@ -4172,7 +4196,7 @@
       <x:c r="A15" s="3">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B15" s="3">
+      <x:c r="B15" s="3" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C15" s="2" t="s">
@@ -4190,8 +4214,8 @@
       <x:c r="G15" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H15" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H15" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I15" s="56">
         <x:v>46197</x:v>
@@ -4239,7 +4263,7 @@
       <x:c r="A16" s="7">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B16" s="7">
+      <x:c r="B16" s="7" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C16" s="8" t="s">
@@ -4257,8 +4281,8 @@
       <x:c r="G16" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H16" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H16" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I16" s="55">
         <x:v>46197</x:v>
@@ -4306,7 +4330,7 @@
       <x:c r="A17" s="3">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B17" s="3">
+      <x:c r="B17" s="3" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="C17" s="2" t="s">
@@ -4324,8 +4348,8 @@
       <x:c r="G17" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H17" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H17" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I17" s="56">
         <x:v>46197</x:v>
@@ -4373,7 +4397,7 @@
       <x:c r="A18" s="7">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B18" s="7">
+      <x:c r="B18" s="7" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="8" t="s">
@@ -4391,8 +4415,8 @@
       <x:c r="G18" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H18" s="7" t="s">
-        <x:v>13</x:v>
+      <x:c r="H18" s="7" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I18" s="55">
         <x:v>46196</x:v>
@@ -4465,7 +4489,7 @@
       <x:c r="A20" s="3">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B20" s="3">
+      <x:c r="B20" s="3" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C20" s="2" t="s">
@@ -4483,8 +4507,8 @@
       <x:c r="G20" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H20" s="3" t="s">
-        <x:v>13</x:v>
+      <x:c r="H20" s="3" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I20" s="56">
         <x:v>46196</x:v>
@@ -4532,7 +4556,7 @@
       <x:c r="A21" s="7">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B21" s="7">
+      <x:c r="B21" s="7" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="C21" s="8" t="s">
@@ -4550,8 +4574,8 @@
       <x:c r="G21" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H21" s="7" t="s">
-        <x:v>13</x:v>
+      <x:c r="H21" s="7" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I21" s="55">
         <x:v>46196</x:v>
@@ -4599,7 +4623,7 @@
       <x:c r="A22" s="3">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B22" s="3">
+      <x:c r="B22" s="3" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="C22" s="2" t="s">
@@ -4617,8 +4641,8 @@
       <x:c r="G22" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H22" s="3" t="s">
-        <x:v>13</x:v>
+      <x:c r="H22" s="3" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I22" s="56">
         <x:v>46196</x:v>
@@ -4666,7 +4690,7 @@
       <x:c r="A23" s="7">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B23" s="7">
+      <x:c r="B23" s="7" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="C23" s="8" t="s">
@@ -4684,8 +4708,8 @@
       <x:c r="G23" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H23" s="7" t="s">
-        <x:v>13</x:v>
+      <x:c r="H23" s="7" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I23" s="55">
         <x:v>46196</x:v>
@@ -4733,7 +4757,7 @@
       <x:c r="A24" s="3">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B24" s="3">
+      <x:c r="B24" s="3" t="n">
         <x:v>13</x:v>
       </x:c>
       <x:c r="C24" s="2" t="s">
@@ -4751,8 +4775,8 @@
       <x:c r="G24" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H24" s="3" t="s">
-        <x:v>13</x:v>
+      <x:c r="H24" s="3" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I24" s="56">
         <x:v>46196</x:v>
@@ -4800,7 +4824,7 @@
       <x:c r="A25" s="7">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B25" s="7">
+      <x:c r="B25" s="7" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="C25" s="8" t="s">
@@ -4818,8 +4842,8 @@
       <x:c r="G25" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H25" s="7" t="s">
-        <x:v>13</x:v>
+      <x:c r="H25" s="7" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I25" s="55">
         <x:v>46196</x:v>
@@ -4867,7 +4891,7 @@
       <x:c r="A26" s="3">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B26" s="3">
+      <x:c r="B26" s="3" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="C26" s="2" t="s">
@@ -4885,8 +4909,8 @@
       <x:c r="G26" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H26" s="3" t="s">
-        <x:v>13</x:v>
+      <x:c r="H26" s="3" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I26" s="56">
         <x:v>46196</x:v>
@@ -4934,7 +4958,7 @@
       <x:c r="A27" s="7">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B27" s="7">
+      <x:c r="B27" s="7" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="C27" s="8" t="s">
@@ -4952,8 +4976,8 @@
       <x:c r="G27" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H27" s="7" t="s">
-        <x:v>13</x:v>
+      <x:c r="H27" s="7" t="str">
+        <x:v>Day 01</x:v>
       </x:c>
       <x:c r="I27" s="55">
         <x:v>46196</x:v>
@@ -5001,7 +5025,7 @@
       <x:c r="A28" s="3">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B28" s="3">
+      <x:c r="B28" s="3" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="C28" s="2" t="s">
@@ -5019,8 +5043,8 @@
       <x:c r="G28" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H28" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H28" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I28" s="56">
         <x:v>46197</x:v>
@@ -5093,7 +5117,7 @@
       <x:c r="A30" s="7">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B30" s="7">
+      <x:c r="B30" s="7" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="C30" s="8" t="s">
@@ -5111,8 +5135,8 @@
       <x:c r="G30" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H30" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H30" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I30" s="55">
         <x:v>46197</x:v>
@@ -5160,7 +5184,7 @@
       <x:c r="A31" s="3">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B31" s="3">
+      <x:c r="B31" s="3" t="n">
         <x:v>19</x:v>
       </x:c>
       <x:c r="C31" s="2" t="s">
@@ -5178,8 +5202,8 @@
       <x:c r="G31" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H31" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H31" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I31" s="56">
         <x:v>46197</x:v>
@@ -5227,7 +5251,7 @@
       <x:c r="A32" s="7">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B32" s="7">
+      <x:c r="B32" s="7" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="C32" s="8" t="s">
@@ -5245,8 +5269,8 @@
       <x:c r="G32" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H32" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H32" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I32" s="55">
         <x:v>46197</x:v>
@@ -5294,7 +5318,7 @@
       <x:c r="A33" s="3">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B33" s="3">
+      <x:c r="B33" s="3" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="C33" s="2" t="s">
@@ -5312,8 +5336,8 @@
       <x:c r="G33" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H33" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H33" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I33" s="56">
         <x:v>46197</x:v>
@@ -5361,7 +5385,7 @@
       <x:c r="A34" s="7">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B34" s="7">
+      <x:c r="B34" s="7" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="C34" s="8" t="s">
@@ -5379,8 +5403,8 @@
       <x:c r="G34" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H34" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H34" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I34" s="55">
         <x:v>46197</x:v>
@@ -5428,7 +5452,7 @@
       <x:c r="A35" s="3">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B35" s="3">
+      <x:c r="B35" s="3" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="C35" s="2" t="s">
@@ -5446,8 +5470,8 @@
       <x:c r="G35" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H35" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H35" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I35" s="56">
         <x:v>46197</x:v>
@@ -5495,7 +5519,7 @@
       <x:c r="A36" s="7">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B36" s="7">
+      <x:c r="B36" s="7" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="C36" s="8" t="s">
@@ -5513,8 +5537,8 @@
       <x:c r="G36" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H36" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H36" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I36" s="55">
         <x:v>46197</x:v>
@@ -5562,7 +5586,7 @@
       <x:c r="A37" s="3">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B37" s="3">
+      <x:c r="B37" s="3" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="C37" s="2" t="s">
@@ -5580,8 +5604,8 @@
       <x:c r="G37" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H37" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H37" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I37" s="56">
         <x:v>46197</x:v>
@@ -5629,7 +5653,7 @@
       <x:c r="A38" s="7">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B38" s="7">
+      <x:c r="B38" s="7" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="C38" s="8" t="s">
@@ -5647,8 +5671,8 @@
       <x:c r="G38" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H38" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H38" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I38" s="55">
         <x:v>46197</x:v>
@@ -5721,7 +5745,7 @@
       <x:c r="A40" s="3">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B40" s="3">
+      <x:c r="B40" s="3" t="n">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C40" s="2" t="s">
@@ -5739,8 +5763,8 @@
       <x:c r="G40" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H40" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H40" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I40" s="56">
         <x:v>46197</x:v>
@@ -5788,7 +5812,7 @@
       <x:c r="A41" s="7">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B41" s="7">
+      <x:c r="B41" s="7" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="C41" s="8" t="s">
@@ -5806,8 +5830,8 @@
       <x:c r="G41" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H41" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H41" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I41" s="55">
         <x:v>46197</x:v>
@@ -5855,7 +5879,7 @@
       <x:c r="A42" s="3">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B42" s="3">
+      <x:c r="B42" s="3" t="n">
         <x:v>29</x:v>
       </x:c>
       <x:c r="C42" s="2" t="s">
@@ -5873,8 +5897,8 @@
       <x:c r="G42" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H42" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H42" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I42" s="56">
         <x:v>46197</x:v>
@@ -5922,7 +5946,7 @@
       <x:c r="A43" s="7">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B43" s="7">
+      <x:c r="B43" s="7" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="C43" s="8" t="s">
@@ -5940,8 +5964,8 @@
       <x:c r="G43" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H43" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H43" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I43" s="55">
         <x:v>46197</x:v>
@@ -5989,7 +6013,7 @@
       <x:c r="A44" s="3">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B44" s="3">
+      <x:c r="B44" s="3" t="n">
         <x:v>31</x:v>
       </x:c>
       <x:c r="C44" s="2" t="s">
@@ -6007,8 +6031,8 @@
       <x:c r="G44" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H44" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H44" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I44" s="56">
         <x:v>46197</x:v>
@@ -6056,7 +6080,7 @@
       <x:c r="A45" s="7">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="B45" s="7">
+      <x:c r="B45" s="7" t="n">
         <x:v>32</x:v>
       </x:c>
       <x:c r="C45" s="8" t="s">
@@ -6074,8 +6098,8 @@
       <x:c r="G45" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H45" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H45" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I45" s="55">
         <x:v>46197</x:v>
@@ -6123,7 +6147,7 @@
       <x:c r="A46" s="3">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B46" s="3">
+      <x:c r="B46" s="3" t="n">
         <x:v>33</x:v>
       </x:c>
       <x:c r="C46" s="2" t="s">
@@ -6141,8 +6165,8 @@
       <x:c r="G46" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H46" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H46" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I46" s="56">
         <x:v>46197</x:v>
@@ -6190,7 +6214,7 @@
       <x:c r="A47" s="7">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="B47" s="7">
+      <x:c r="B47" s="7" t="n">
         <x:v>34</x:v>
       </x:c>
       <x:c r="C47" s="8" t="s">
@@ -6208,8 +6232,8 @@
       <x:c r="G47" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H47" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H47" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I47" s="55">
         <x:v>46197</x:v>
@@ -6282,7 +6306,7 @@
       <x:c r="A49" s="3">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B49" s="3">
+      <x:c r="B49" s="3" t="n">
         <x:v>35</x:v>
       </x:c>
       <x:c r="C49" s="2" t="s">
@@ -6300,8 +6324,8 @@
       <x:c r="G49" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H49" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H49" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I49" s="56">
         <x:v>46197</x:v>
@@ -6349,7 +6373,7 @@
       <x:c r="A50" s="7">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="B50" s="7">
+      <x:c r="B50" s="7" t="n">
         <x:v>36</x:v>
       </x:c>
       <x:c r="C50" s="8" t="s">
@@ -6367,8 +6391,8 @@
       <x:c r="G50" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H50" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H50" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I50" s="55">
         <x:v>46197</x:v>
@@ -6416,7 +6440,7 @@
       <x:c r="A51" s="3">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B51" s="3">
+      <x:c r="B51" s="3" t="n">
         <x:v>37</x:v>
       </x:c>
       <x:c r="C51" s="2" t="s">
@@ -6434,8 +6458,8 @@
       <x:c r="G51" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H51" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H51" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I51" s="56">
         <x:v>46197</x:v>
@@ -6483,7 +6507,7 @@
       <x:c r="A52" s="7">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="B52" s="7">
+      <x:c r="B52" s="7" t="n">
         <x:v>38</x:v>
       </x:c>
       <x:c r="C52" s="8" t="s">
@@ -6501,8 +6525,8 @@
       <x:c r="G52" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H52" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H52" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I52" s="55">
         <x:v>46197</x:v>
@@ -6550,7 +6574,7 @@
       <x:c r="A53" s="3">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B53" s="3">
+      <x:c r="B53" s="3" t="n">
         <x:v>39</x:v>
       </x:c>
       <x:c r="C53" s="2" t="s">
@@ -6568,8 +6592,8 @@
       <x:c r="G53" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H53" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H53" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I53" s="56">
         <x:v>46197</x:v>
@@ -6617,7 +6641,7 @@
       <x:c r="A54" s="7">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B54" s="7">
+      <x:c r="B54" s="7" t="n">
         <x:v>40</x:v>
       </x:c>
       <x:c r="C54" s="8" t="s">
@@ -6635,8 +6659,8 @@
       <x:c r="G54" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H54" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H54" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I54" s="55">
         <x:v>46197</x:v>
@@ -6684,7 +6708,7 @@
       <x:c r="A55" s="3">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="B55" s="3">
+      <x:c r="B55" s="3" t="n">
         <x:v>41</x:v>
       </x:c>
       <x:c r="C55" s="2" t="s">
@@ -6702,8 +6726,8 @@
       <x:c r="G55" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H55" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H55" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I55" s="56">
         <x:v>46198</x:v>
@@ -6801,7 +6825,7 @@
       <x:c r="A58" s="7">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="B58" s="7">
+      <x:c r="B58" s="7" t="n">
         <x:v>42</x:v>
       </x:c>
       <x:c r="C58" s="8" t="s">
@@ -6819,8 +6843,8 @@
       <x:c r="G58" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H58" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H58" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I58" s="55">
         <x:v>46197</x:v>
@@ -6868,7 +6892,7 @@
       <x:c r="A59" s="3">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B59" s="3">
+      <x:c r="B59" s="3" t="n">
         <x:v>43</x:v>
       </x:c>
       <x:c r="C59" s="2" t="s">
@@ -6886,8 +6910,8 @@
       <x:c r="G59" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H59" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H59" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I59" s="56">
         <x:v>46197</x:v>
@@ -6935,7 +6959,7 @@
       <x:c r="A60" s="7">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="B60" s="7">
+      <x:c r="B60" s="7" t="n">
         <x:v>44</x:v>
       </x:c>
       <x:c r="C60" s="8" t="s">
@@ -6953,8 +6977,8 @@
       <x:c r="G60" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H60" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H60" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I60" s="55">
         <x:v>46197</x:v>
@@ -7002,7 +7026,7 @@
       <x:c r="A61" s="3">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B61" s="3">
+      <x:c r="B61" s="3" t="n">
         <x:v>45</x:v>
       </x:c>
       <x:c r="C61" s="2" t="s">
@@ -7020,8 +7044,8 @@
       <x:c r="G61" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H61" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H61" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I61" s="56">
         <x:v>46197</x:v>
@@ -7069,7 +7093,7 @@
       <x:c r="A62" s="7">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="B62" s="7">
+      <x:c r="B62" s="7" t="n">
         <x:v>46</x:v>
       </x:c>
       <x:c r="C62" s="8" t="s">
@@ -7087,8 +7111,8 @@
       <x:c r="G62" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H62" s="7" t="s">
-        <x:v>16</x:v>
+      <x:c r="H62" s="7" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I62" s="55">
         <x:v>46197</x:v>
@@ -7136,7 +7160,7 @@
       <x:c r="A63" s="3">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="B63" s="3">
+      <x:c r="B63" s="3" t="n">
         <x:v>47</x:v>
       </x:c>
       <x:c r="C63" s="2" t="s">
@@ -7154,8 +7178,8 @@
       <x:c r="G63" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H63" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H63" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I63" s="56">
         <x:v>46198</x:v>
@@ -7203,7 +7227,7 @@
       <x:c r="A64" s="7">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="B64" s="7">
+      <x:c r="B64" s="7" t="n">
         <x:v>48</x:v>
       </x:c>
       <x:c r="C64" s="8" t="s">
@@ -7221,8 +7245,8 @@
       <x:c r="G64" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H64" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H64" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I64" s="55">
         <x:v>46198</x:v>
@@ -7270,7 +7294,7 @@
       <x:c r="A65" s="3">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B65" s="3">
+      <x:c r="B65" s="3" t="n">
         <x:v>49</x:v>
       </x:c>
       <x:c r="C65" s="2" t="s">
@@ -7288,8 +7312,8 @@
       <x:c r="G65" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H65" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H65" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I65" s="56">
         <x:v>46198</x:v>
@@ -7337,7 +7361,7 @@
       <x:c r="A66" s="7">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="B66" s="7">
+      <x:c r="B66" s="7" t="n">
         <x:v>50</x:v>
       </x:c>
       <x:c r="C66" s="8" t="s">
@@ -7355,8 +7379,8 @@
       <x:c r="G66" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H66" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H66" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I66" s="55">
         <x:v>46198</x:v>
@@ -7404,7 +7428,7 @@
       <x:c r="A67" s="3">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="B67" s="3">
+      <x:c r="B67" s="3" t="n">
         <x:v>51</x:v>
       </x:c>
       <x:c r="C67" s="2" t="s">
@@ -7422,8 +7446,8 @@
       <x:c r="G67" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H67" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H67" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I67" s="56">
         <x:v>46198</x:v>
@@ -7471,7 +7495,7 @@
       <x:c r="A68" s="7">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="B68" s="7">
+      <x:c r="B68" s="7" t="n">
         <x:v>52</x:v>
       </x:c>
       <x:c r="C68" s="8" t="s">
@@ -7489,8 +7513,8 @@
       <x:c r="G68" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H68" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H68" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I68" s="55">
         <x:v>46198</x:v>
@@ -7538,7 +7562,7 @@
       <x:c r="A69" s="3">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="B69" s="3">
+      <x:c r="B69" s="3" t="n">
         <x:v>53</x:v>
       </x:c>
       <x:c r="C69" s="2" t="s">
@@ -7556,8 +7580,8 @@
       <x:c r="G69" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H69" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H69" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I69" s="56">
         <x:v>46198</x:v>
@@ -7605,7 +7629,7 @@
       <x:c r="A70" s="7">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="B70" s="7">
+      <x:c r="B70" s="7" t="n">
         <x:v>54</x:v>
       </x:c>
       <x:c r="C70" s="8" t="s">
@@ -7623,8 +7647,8 @@
       <x:c r="G70" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H70" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H70" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I70" s="55">
         <x:v>46198</x:v>
@@ -7672,7 +7696,7 @@
       <x:c r="A71" s="3">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="B71" s="3">
+      <x:c r="B71" s="3" t="n">
         <x:v>55</x:v>
       </x:c>
       <x:c r="C71" s="2" t="s">
@@ -7690,8 +7714,8 @@
       <x:c r="G71" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H71" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H71" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I71" s="56">
         <x:v>46198</x:v>
@@ -7739,7 +7763,7 @@
       <x:c r="A72" s="7">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="B72" s="7">
+      <x:c r="B72" s="7" t="n">
         <x:v>56</x:v>
       </x:c>
       <x:c r="C72" s="8" t="s">
@@ -7757,8 +7781,8 @@
       <x:c r="G72" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H72" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H72" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I72" s="55">
         <x:v>46198</x:v>
@@ -7806,7 +7830,7 @@
       <x:c r="A73" s="3">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="B73" s="3">
+      <x:c r="B73" s="3" t="n">
         <x:v>57</x:v>
       </x:c>
       <x:c r="C73" s="2" t="s">
@@ -7824,8 +7848,8 @@
       <x:c r="G73" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H73" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H73" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I73" s="56">
         <x:v>46198</x:v>
@@ -7873,7 +7897,7 @@
       <x:c r="A74" s="7">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="B74" s="7">
+      <x:c r="B74" s="7" t="n">
         <x:v>58</x:v>
       </x:c>
       <x:c r="C74" s="8" t="s">
@@ -7891,8 +7915,8 @@
       <x:c r="G74" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H74" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H74" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I74" s="55">
         <x:v>46198</x:v>
@@ -7965,7 +7989,7 @@
       <x:c r="A76" s="3">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="B76" s="3">
+      <x:c r="B76" s="3" t="n">
         <x:v>59</x:v>
       </x:c>
       <x:c r="C76" s="2" t="s">
@@ -7983,8 +8007,8 @@
       <x:c r="G76" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H76" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H76" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I76" s="56">
         <x:v>46198</x:v>
@@ -8032,7 +8056,7 @@
       <x:c r="A77" s="7">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="B77" s="7">
+      <x:c r="B77" s="7" t="n">
         <x:v>60</x:v>
       </x:c>
       <x:c r="C77" s="8" t="s">
@@ -8050,8 +8074,8 @@
       <x:c r="G77" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H77" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H77" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I77" s="55">
         <x:v>46198</x:v>
@@ -8099,7 +8123,7 @@
       <x:c r="A78" s="3">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="B78" s="3">
+      <x:c r="B78" s="3" t="n">
         <x:v>61</x:v>
       </x:c>
       <x:c r="C78" s="2" t="s">
@@ -8117,8 +8141,8 @@
       <x:c r="G78" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H78" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H78" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I78" s="56">
         <x:v>46198</x:v>
@@ -8166,7 +8190,7 @@
       <x:c r="A79" s="7">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="B79" s="7">
+      <x:c r="B79" s="7" t="n">
         <x:v>62</x:v>
       </x:c>
       <x:c r="C79" s="8" t="s">
@@ -8184,8 +8208,8 @@
       <x:c r="G79" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H79" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H79" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I79" s="55">
         <x:v>46198</x:v>
@@ -8233,7 +8257,7 @@
       <x:c r="A80" s="3">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="B80" s="3">
+      <x:c r="B80" s="3" t="n">
         <x:v>63</x:v>
       </x:c>
       <x:c r="C80" s="2" t="s">
@@ -8251,8 +8275,8 @@
       <x:c r="G80" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H80" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H80" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I80" s="56">
         <x:v>46198</x:v>
@@ -8325,7 +8349,7 @@
       <x:c r="A82" s="7">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="B82" s="7">
+      <x:c r="B82" s="7" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="C82" s="8" t="s">
@@ -8343,8 +8367,8 @@
       <x:c r="G82" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H82" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H82" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I82" s="55">
         <x:v>46198</x:v>
@@ -8392,7 +8416,7 @@
       <x:c r="A83" s="3">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="B83" s="3">
+      <x:c r="B83" s="3" t="n">
         <x:v>65</x:v>
       </x:c>
       <x:c r="C83" s="2" t="s">
@@ -8410,8 +8434,8 @@
       <x:c r="G83" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H83" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="H83" s="3" t="str">
+        <x:v>Day 02</x:v>
       </x:c>
       <x:c r="I83" s="56">
         <x:v>46197</x:v>
@@ -8459,7 +8483,7 @@
       <x:c r="A84" s="7">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="B84" s="7">
+      <x:c r="B84" s="7" t="n">
         <x:v>66</x:v>
       </x:c>
       <x:c r="C84" s="8" t="s">
@@ -8477,8 +8501,8 @@
       <x:c r="G84" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H84" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H84" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I84" s="55">
         <x:v>46198</x:v>
@@ -8526,7 +8550,7 @@
       <x:c r="A85" s="3">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="B85" s="3">
+      <x:c r="B85" s="3" t="n">
         <x:v>67</x:v>
       </x:c>
       <x:c r="C85" s="2" t="s">
@@ -8544,8 +8568,8 @@
       <x:c r="G85" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H85" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H85" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I85" s="56">
         <x:v>46198</x:v>
@@ -8593,7 +8617,7 @@
       <x:c r="A86" s="7">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="B86" s="7">
+      <x:c r="B86" s="7" t="n">
         <x:v>68</x:v>
       </x:c>
       <x:c r="C86" s="8" t="s">
@@ -8611,8 +8635,8 @@
       <x:c r="G86" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H86" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H86" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I86" s="55">
         <x:v>46198</x:v>
@@ -8660,7 +8684,7 @@
       <x:c r="A87" s="3">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="B87" s="3">
+      <x:c r="B87" s="3" t="n">
         <x:v>69</x:v>
       </x:c>
       <x:c r="C87" s="2" t="s">
@@ -8678,8 +8702,8 @@
       <x:c r="G87" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H87" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H87" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I87" s="56">
         <x:v>46198</x:v>
@@ -8727,7 +8751,7 @@
       <x:c r="A88" s="7">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="B88" s="7">
+      <x:c r="B88" s="7" t="n">
         <x:v>70</x:v>
       </x:c>
       <x:c r="C88" s="8" t="s">
@@ -8745,8 +8769,8 @@
       <x:c r="G88" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H88" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H88" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I88" s="55">
         <x:v>46198</x:v>
@@ -8819,7 +8843,7 @@
       <x:c r="A90" s="3">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="B90" s="3">
+      <x:c r="B90" s="3" t="n">
         <x:v>71</x:v>
       </x:c>
       <x:c r="C90" s="2" t="s">
@@ -8837,8 +8861,8 @@
       <x:c r="G90" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H90" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H90" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I90" s="56">
         <x:v>46198</x:v>
@@ -8886,7 +8910,7 @@
       <x:c r="A91" s="7">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="B91" s="7">
+      <x:c r="B91" s="7" t="n">
         <x:v>72</x:v>
       </x:c>
       <x:c r="C91" s="8" t="s">
@@ -8904,8 +8928,8 @@
       <x:c r="G91" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H91" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H91" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I91" s="55">
         <x:v>46198</x:v>
@@ -8953,7 +8977,7 @@
       <x:c r="A92" s="3">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="B92" s="3">
+      <x:c r="B92" s="3" t="n">
         <x:v>73</x:v>
       </x:c>
       <x:c r="C92" s="2" t="s">
@@ -8971,8 +8995,8 @@
       <x:c r="G92" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H92" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H92" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I92" s="56">
         <x:v>46198</x:v>
@@ -9020,7 +9044,7 @@
       <x:c r="A93" s="7">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="B93" s="7">
+      <x:c r="B93" s="7" t="n">
         <x:v>74</x:v>
       </x:c>
       <x:c r="C93" s="8" t="s">
@@ -9038,8 +9062,8 @@
       <x:c r="G93" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H93" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H93" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I93" s="55">
         <x:v>46198</x:v>
@@ -9087,7 +9111,7 @@
       <x:c r="A94" s="3">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="B94" s="3">
+      <x:c r="B94" s="3" t="n">
         <x:v>75</x:v>
       </x:c>
       <x:c r="C94" s="2" t="s">
@@ -9105,8 +9129,8 @@
       <x:c r="G94" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H94" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H94" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I94" s="56">
         <x:v>46198</x:v>
@@ -9154,7 +9178,7 @@
       <x:c r="A95" s="7">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="B95" s="7">
+      <x:c r="B95" s="7" t="n">
         <x:v>76</x:v>
       </x:c>
       <x:c r="C95" s="8" t="s">
@@ -9172,8 +9196,8 @@
       <x:c r="G95" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H95" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H95" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I95" s="55">
         <x:v>46198</x:v>
@@ -9221,7 +9245,7 @@
       <x:c r="A96" s="3">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="B96" s="3">
+      <x:c r="B96" s="3" t="n">
         <x:v>77</x:v>
       </x:c>
       <x:c r="C96" s="2" t="s">
@@ -9239,8 +9263,8 @@
       <x:c r="G96" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H96" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H96" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I96" s="56">
         <x:v>46198</x:v>
@@ -9288,7 +9312,7 @@
       <x:c r="A97" s="7">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="B97" s="7">
+      <x:c r="B97" s="7" t="n">
         <x:v>78</x:v>
       </x:c>
       <x:c r="C97" s="8" t="s">
@@ -9306,8 +9330,8 @@
       <x:c r="G97" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H97" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H97" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I97" s="55">
         <x:v>46198</x:v>
@@ -9380,7 +9404,7 @@
       <x:c r="A99" s="3">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="B99" s="3">
+      <x:c r="B99" s="3" t="n">
         <x:v>79</x:v>
       </x:c>
       <x:c r="C99" s="2" t="s">
@@ -9398,8 +9422,8 @@
       <x:c r="G99" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H99" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H99" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I99" s="56">
         <x:v>46198</x:v>
@@ -9447,7 +9471,7 @@
       <x:c r="A100" s="7">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="B100" s="7">
+      <x:c r="B100" s="7" t="n">
         <x:v>80</x:v>
       </x:c>
       <x:c r="C100" s="8" t="s">
@@ -9465,8 +9489,8 @@
       <x:c r="G100" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H100" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H100" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I100" s="55">
         <x:v>46198</x:v>
@@ -9514,7 +9538,7 @@
       <x:c r="A101" s="3">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="B101" s="3">
+      <x:c r="B101" s="3" t="n">
         <x:v>81</x:v>
       </x:c>
       <x:c r="C101" s="2" t="s">
@@ -9532,8 +9556,8 @@
       <x:c r="G101" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H101" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H101" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I101" s="56">
         <x:v>46198</x:v>
@@ -9581,7 +9605,7 @@
       <x:c r="A102" s="7">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="B102" s="7">
+      <x:c r="B102" s="7" t="n">
         <x:v>82</x:v>
       </x:c>
       <x:c r="C102" s="8" t="s">
@@ -9599,8 +9623,8 @@
       <x:c r="G102" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H102" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H102" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I102" s="55">
         <x:v>46198</x:v>
@@ -9648,7 +9672,7 @@
       <x:c r="A103" s="3">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B103" s="3">
+      <x:c r="B103" s="3" t="n">
         <x:v>83</x:v>
       </x:c>
       <x:c r="C103" s="2" t="s">
@@ -9666,8 +9690,8 @@
       <x:c r="G103" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H103" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H103" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I103" s="56">
         <x:v>46198</x:v>
@@ -9715,7 +9739,7 @@
       <x:c r="A104" s="7">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="B104" s="7">
+      <x:c r="B104" s="7" t="n">
         <x:v>84</x:v>
       </x:c>
       <x:c r="C104" s="8" t="s">
@@ -9733,8 +9757,8 @@
       <x:c r="G104" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H104" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H104" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I104" s="55">
         <x:v>46198</x:v>
@@ -9782,7 +9806,7 @@
       <x:c r="A105" s="3">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="B105" s="3">
+      <x:c r="B105" s="3" t="n">
         <x:v>85</x:v>
       </x:c>
       <x:c r="C105" s="2" t="s">
@@ -9800,8 +9824,8 @@
       <x:c r="G105" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H105" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H105" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I105" s="56">
         <x:v>46198</x:v>
@@ -9849,7 +9873,7 @@
       <x:c r="A106" s="7">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="B106" s="7">
+      <x:c r="B106" s="7" t="n">
         <x:v>86</x:v>
       </x:c>
       <x:c r="C106" s="8" t="s">
@@ -9867,8 +9891,8 @@
       <x:c r="G106" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H106" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H106" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I106" s="55">
         <x:v>46198</x:v>
@@ -9916,7 +9940,7 @@
       <x:c r="A107" s="3">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="B107" s="3">
+      <x:c r="B107" s="3" t="n">
         <x:v>87</x:v>
       </x:c>
       <x:c r="C107" s="2" t="s">
@@ -9934,8 +9958,8 @@
       <x:c r="G107" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H107" s="3" t="s">
-        <x:v>19</x:v>
+      <x:c r="H107" s="3" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I107" s="56">
         <x:v>46198</x:v>
@@ -9983,7 +10007,7 @@
       <x:c r="A108" s="7">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B108" s="7">
+      <x:c r="B108" s="7" t="n">
         <x:v>88</x:v>
       </x:c>
       <x:c r="C108" s="8" t="s">
@@ -10001,8 +10025,8 @@
       <x:c r="G108" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H108" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="H108" s="7" t="str">
+        <x:v>Day 03</x:v>
       </x:c>
       <x:c r="I108" s="55">
         <x:v>46198</x:v>
@@ -10050,7 +10074,7 @@
       <x:c r="A109" s="3">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="B109" s="3">
+      <x:c r="B109" s="3" t="n">
         <x:v>89</x:v>
       </x:c>
       <x:c r="C109" s="2" t="s">
@@ -10068,8 +10092,8 @@
       <x:c r="G109" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H109" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="H109" s="3" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I109" s="56">
         <x:v>46199</x:v>
@@ -10117,7 +10141,7 @@
       <x:c r="A110" s="7">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="B110" s="7">
+      <x:c r="B110" s="7" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C110" s="8" t="s">
@@ -10135,8 +10159,8 @@
       <x:c r="G110" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H110" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="H110" s="7" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I110" s="55">
         <x:v>46199</x:v>
@@ -10184,7 +10208,7 @@
       <x:c r="A111" s="3">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="B111" s="3">
+      <x:c r="B111" s="3" t="n">
         <x:v>91</x:v>
       </x:c>
       <x:c r="C111" s="2" t="s">
@@ -10202,8 +10226,8 @@
       <x:c r="G111" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H111" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="H111" s="3" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I111" s="56">
         <x:v>46199</x:v>
@@ -10251,7 +10275,7 @@
       <x:c r="A112" s="7">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="B112" s="7">
+      <x:c r="B112" s="7" t="n">
         <x:v>92</x:v>
       </x:c>
       <x:c r="C112" s="8" t="s">
@@ -10269,8 +10293,8 @@
       <x:c r="G112" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H112" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="H112" s="7" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I112" s="55">
         <x:v>46199</x:v>
@@ -10318,7 +10342,7 @@
       <x:c r="A113" s="3">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="B113" s="3">
+      <x:c r="B113" s="3" t="n">
         <x:v>93</x:v>
       </x:c>
       <x:c r="C113" s="2" t="s">
@@ -10336,8 +10360,8 @@
       <x:c r="G113" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H113" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="H113" s="3" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I113" s="56">
         <x:v>46199</x:v>
@@ -10385,7 +10409,7 @@
       <x:c r="A114" s="7">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="B114" s="7">
+      <x:c r="B114" s="7" t="n">
         <x:v>94</x:v>
       </x:c>
       <x:c r="C114" s="8" t="s">
@@ -10403,8 +10427,8 @@
       <x:c r="G114" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H114" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="H114" s="7" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I114" s="55">
         <x:v>46199</x:v>
@@ -10452,7 +10476,7 @@
       <x:c r="A115" s="3">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="B115" s="3">
+      <x:c r="B115" s="3" t="n">
         <x:v>95</x:v>
       </x:c>
       <x:c r="C115" s="2" t="s">
@@ -10470,8 +10494,8 @@
       <x:c r="G115" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H115" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="H115" s="3" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I115" s="56">
         <x:v>46199</x:v>
@@ -10519,7 +10543,7 @@
       <x:c r="A116" s="7">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="B116" s="7">
+      <x:c r="B116" s="7" t="n">
         <x:v>96</x:v>
       </x:c>
       <x:c r="C116" s="8" t="s">
@@ -10537,8 +10561,8 @@
       <x:c r="G116" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H116" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="H116" s="7" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I116" s="55">
         <x:v>46199</x:v>
@@ -10611,7 +10635,7 @@
       <x:c r="A118" s="3">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="B118" s="3">
+      <x:c r="B118" s="3" t="n">
         <x:v>97</x:v>
       </x:c>
       <x:c r="C118" s="2" t="s">
@@ -10629,8 +10653,8 @@
       <x:c r="G118" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H118" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="H118" s="3" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I118" s="56">
         <x:v>46199</x:v>
@@ -10678,7 +10702,7 @@
       <x:c r="A119" s="7">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="B119" s="7">
+      <x:c r="B119" s="7" t="n">
         <x:v>98</x:v>
       </x:c>
       <x:c r="C119" s="8" t="s">
@@ -10696,8 +10720,8 @@
       <x:c r="G119" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H119" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="H119" s="7" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I119" s="55">
         <x:v>46199</x:v>
@@ -10745,7 +10769,7 @@
       <x:c r="A120" s="3">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="B120" s="3">
+      <x:c r="B120" s="3" t="n">
         <x:v>99</x:v>
       </x:c>
       <x:c r="C120" s="2" t="s">
@@ -10763,8 +10787,8 @@
       <x:c r="G120" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H120" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="H120" s="3" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I120" s="56">
         <x:v>46199</x:v>
@@ -10812,7 +10836,7 @@
       <x:c r="A121" s="7">
         <x:v>102</x:v>
       </x:c>
-      <x:c r="B121" s="7">
+      <x:c r="B121" s="7" t="n">
         <x:v>100</x:v>
       </x:c>
       <x:c r="C121" s="8" t="s">
@@ -10830,8 +10854,8 @@
       <x:c r="G121" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H121" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="H121" s="7" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I121" s="55">
         <x:v>46199</x:v>
@@ -10879,7 +10903,7 @@
       <x:c r="A122" s="3">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="B122" s="3">
+      <x:c r="B122" s="3" t="n">
         <x:v>143</x:v>
       </x:c>
       <x:c r="C122" s="2" t="s">
@@ -10897,8 +10921,8 @@
       <x:c r="G122" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H122" s="3" t="s">
-        <x:v>30</x:v>
+      <x:c r="H122" s="3" t="str">
+        <x:v>Day 08</x:v>
       </x:c>
       <x:c r="I122" s="56">
         <x:v>46203</x:v>
@@ -10946,7 +10970,7 @@
       <x:c r="A123" s="7">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="B123" s="7">
+      <x:c r="B123" s="7" t="n">
         <x:v>144</x:v>
       </x:c>
       <x:c r="C123" s="8" t="s">
@@ -10964,8 +10988,8 @@
       <x:c r="G123" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H123" s="7" t="s">
-        <x:v>32</x:v>
+      <x:c r="H123" s="7" t="str">
+        <x:v>Day 09</x:v>
       </x:c>
       <x:c r="I123" s="55">
         <x:v>46205</x:v>
@@ -11013,7 +11037,7 @@
       <x:c r="A124" s="3">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="B124" s="3">
+      <x:c r="B124" s="3" t="n">
         <x:v>145</x:v>
       </x:c>
       <x:c r="C124" s="2" t="s">
@@ -11031,8 +11055,8 @@
       <x:c r="G124" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H124" s="3" t="s">
-        <x:v>32</x:v>
+      <x:c r="H124" s="3" t="str">
+        <x:v>Day 09</x:v>
       </x:c>
       <x:c r="I124" s="56">
         <x:v>46205</x:v>
@@ -11080,7 +11104,7 @@
       <x:c r="A125" s="7">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="B125" s="7">
+      <x:c r="B125" s="7" t="n">
         <x:v>146</x:v>
       </x:c>
       <x:c r="C125" s="8" t="s">
@@ -11098,8 +11122,8 @@
       <x:c r="G125" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H125" s="7" t="s">
-        <x:v>32</x:v>
+      <x:c r="H125" s="7" t="str">
+        <x:v>Day 09</x:v>
       </x:c>
       <x:c r="I125" s="55">
         <x:v>46205</x:v>
@@ -11172,7 +11196,7 @@
       <x:c r="A127" s="3">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="B127" s="3">
+      <x:c r="B127" s="3" t="n">
         <x:v>101</x:v>
       </x:c>
       <x:c r="C127" s="2" t="s">
@@ -11190,8 +11214,8 @@
       <x:c r="G127" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H127" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="H127" s="3" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I127" s="56">
         <x:v>46199</x:v>
@@ -11239,7 +11263,7 @@
       <x:c r="A128" s="7">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="B128" s="7">
+      <x:c r="B128" s="7" t="n">
         <x:v>102</x:v>
       </x:c>
       <x:c r="C128" s="8" t="s">
@@ -11257,8 +11281,8 @@
       <x:c r="G128" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H128" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="H128" s="7" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I128" s="55">
         <x:v>46199</x:v>
@@ -11306,7 +11330,7 @@
       <x:c r="A129" s="3">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="B129" s="3">
+      <x:c r="B129" s="3" t="n">
         <x:v>103</x:v>
       </x:c>
       <x:c r="C129" s="2" t="s">
@@ -11324,8 +11348,8 @@
       <x:c r="G129" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H129" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="H129" s="3" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I129" s="56">
         <x:v>46199</x:v>
@@ -11373,7 +11397,7 @@
       <x:c r="A130" s="7">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="B130" s="7">
+      <x:c r="B130" s="7" t="n">
         <x:v>104</x:v>
       </x:c>
       <x:c r="C130" s="8" t="s">
@@ -11391,8 +11415,8 @@
       <x:c r="G130" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H130" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="H130" s="7" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I130" s="55">
         <x:v>46199</x:v>
@@ -11440,7 +11464,7 @@
       <x:c r="A131" s="3">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="B131" s="3">
+      <x:c r="B131" s="3" t="n">
         <x:v>105</x:v>
       </x:c>
       <x:c r="C131" s="2" t="s">
@@ -11458,8 +11482,8 @@
       <x:c r="G131" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H131" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="H131" s="3" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I131" s="56">
         <x:v>46199</x:v>
@@ -11507,7 +11531,7 @@
       <x:c r="A132" s="7">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="B132" s="7">
+      <x:c r="B132" s="7" t="n">
         <x:v>106</x:v>
       </x:c>
       <x:c r="C132" s="8" t="s">
@@ -11525,8 +11549,8 @@
       <x:c r="G132" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H132" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="H132" s="7" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I132" s="55">
         <x:v>46199</x:v>
@@ -11574,7 +11598,7 @@
       <x:c r="A133" s="3">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="B133" s="3">
+      <x:c r="B133" s="3" t="n">
         <x:v>107</x:v>
       </x:c>
       <x:c r="C133" s="2" t="s">
@@ -11592,8 +11616,8 @@
       <x:c r="G133" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H133" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="H133" s="3" t="str">
+        <x:v>Day 04</x:v>
       </x:c>
       <x:c r="I133" s="56">
         <x:v>46199</x:v>
@@ -11641,7 +11665,7 @@
       <x:c r="A134" s="7">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="B134" s="7">
+      <x:c r="B134" s="7" t="n">
         <x:v>108</x:v>
       </x:c>
       <x:c r="C134" s="8" t="s">
@@ -11659,8 +11683,8 @@
       <x:c r="G134" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H134" s="7" t="s">
-        <x:v>23</x:v>
+      <x:c r="H134" s="7" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I134" s="55">
         <x:v>46200</x:v>
@@ -11708,7 +11732,7 @@
       <x:c r="A135" s="3">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="B135" s="3">
+      <x:c r="B135" s="3" t="n">
         <x:v>109</x:v>
       </x:c>
       <x:c r="C135" s="2" t="s">
@@ -11726,8 +11750,8 @@
       <x:c r="G135" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H135" s="3" t="s">
-        <x:v>23</x:v>
+      <x:c r="H135" s="3" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I135" s="56">
         <x:v>46200</x:v>
@@ -11817,7 +11841,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H137" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I137" s="55"/>
       <x:c r="J137" s="7"/>
@@ -11845,7 +11869,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U137" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="34.04999923706055" customHeight="1">
@@ -11869,7 +11893,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H138" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I138" s="56"/>
       <x:c r="J138" s="3"/>
@@ -11897,7 +11921,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U138" s="2" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="139" ht="34.04999923706055" customHeight="1">
@@ -11921,7 +11945,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H139" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I139" s="55"/>
       <x:c r="J139" s="7"/>
@@ -11949,7 +11973,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U139" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="22.049999237060547" customHeight="1">
@@ -11981,7 +12005,7 @@
       <x:c r="A141" s="3">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="B141" s="3">
+      <x:c r="B141" s="3" t="n">
         <x:v>110</x:v>
       </x:c>
       <x:c r="C141" s="2" t="s">
@@ -11999,8 +12023,8 @@
       <x:c r="G141" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H141" s="3" t="s">
-        <x:v>23</x:v>
+      <x:c r="H141" s="3" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I141" s="56">
         <x:v>46200</x:v>
@@ -12048,7 +12072,7 @@
       <x:c r="A142" s="7">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="B142" s="7">
+      <x:c r="B142" s="7" t="n">
         <x:v>111</x:v>
       </x:c>
       <x:c r="C142" s="8" t="s">
@@ -12066,8 +12090,8 @@
       <x:c r="G142" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H142" s="7" t="s">
-        <x:v>23</x:v>
+      <x:c r="H142" s="7" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I142" s="55">
         <x:v>46200</x:v>
@@ -12115,7 +12139,7 @@
       <x:c r="A143" s="3">
         <x:v>121</x:v>
       </x:c>
-      <x:c r="B143" s="3">
+      <x:c r="B143" s="3" t="n">
         <x:v>112</x:v>
       </x:c>
       <x:c r="C143" s="2" t="s">
@@ -12133,8 +12157,8 @@
       <x:c r="G143" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H143" s="3" t="s">
-        <x:v>23</x:v>
+      <x:c r="H143" s="3" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I143" s="56">
         <x:v>46200</x:v>
@@ -12182,7 +12206,7 @@
       <x:c r="A144" s="7">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="B144" s="7">
+      <x:c r="B144" s="7" t="n">
         <x:v>113</x:v>
       </x:c>
       <x:c r="C144" s="8" t="s">
@@ -12200,8 +12224,8 @@
       <x:c r="G144" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H144" s="7" t="s">
-        <x:v>23</x:v>
+      <x:c r="H144" s="7" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I144" s="55">
         <x:v>46200</x:v>
@@ -12249,7 +12273,7 @@
       <x:c r="A145" s="3">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="B145" s="3">
+      <x:c r="B145" s="3" t="n">
         <x:v>114</x:v>
       </x:c>
       <x:c r="C145" s="2" t="s">
@@ -12267,8 +12291,8 @@
       <x:c r="G145" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H145" s="3" t="s">
-        <x:v>23</x:v>
+      <x:c r="H145" s="3" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I145" s="56">
         <x:v>46200</x:v>
@@ -12316,7 +12340,7 @@
       <x:c r="A146" s="7">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="B146" s="7">
+      <x:c r="B146" s="7" t="n">
         <x:v>115</x:v>
       </x:c>
       <x:c r="C146" s="8" t="s">
@@ -12334,8 +12358,8 @@
       <x:c r="G146" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H146" s="7" t="s">
-        <x:v>23</x:v>
+      <x:c r="H146" s="7" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I146" s="55">
         <x:v>46200</x:v>
@@ -12383,7 +12407,7 @@
       <x:c r="A147" s="3">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="B147" s="3">
+      <x:c r="B147" s="3" t="n">
         <x:v>116</x:v>
       </x:c>
       <x:c r="C147" s="2" t="s">
@@ -12401,8 +12425,8 @@
       <x:c r="G147" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H147" s="3" t="s">
-        <x:v>23</x:v>
+      <x:c r="H147" s="3" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I147" s="56">
         <x:v>46200</x:v>
@@ -12450,7 +12474,7 @@
       <x:c r="A148" s="7">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="B148" s="7">
+      <x:c r="B148" s="7" t="n">
         <x:v>117</x:v>
       </x:c>
       <x:c r="C148" s="8" t="s">
@@ -12468,8 +12492,8 @@
       <x:c r="G148" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H148" s="7" t="s">
-        <x:v>23</x:v>
+      <x:c r="H148" s="7" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I148" s="55">
         <x:v>46200</x:v>
@@ -12517,7 +12541,7 @@
       <x:c r="A149" s="3">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="B149" s="3">
+      <x:c r="B149" s="3" t="n">
         <x:v>118</x:v>
       </x:c>
       <x:c r="C149" s="2" t="s">
@@ -12535,8 +12559,8 @@
       <x:c r="G149" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H149" s="3" t="s">
-        <x:v>23</x:v>
+      <x:c r="H149" s="3" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I149" s="56">
         <x:v>46200</x:v>
@@ -12584,7 +12608,7 @@
       <x:c r="A150" s="7">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="B150" s="7">
+      <x:c r="B150" s="7" t="n">
         <x:v>119</x:v>
       </x:c>
       <x:c r="C150" s="8" t="s">
@@ -12602,8 +12626,8 @@
       <x:c r="G150" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H150" s="7" t="s">
-        <x:v>23</x:v>
+      <x:c r="H150" s="7" t="str">
+        <x:v>Day 05</x:v>
       </x:c>
       <x:c r="I150" s="55">
         <x:v>46200</x:v>
@@ -12651,9 +12675,7 @@
       <x:c r="A151" s="3">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="B151" s="3">
-        <x:v>120</x:v>
-      </x:c>
+      <x:c r="B151" s="3"/>
       <x:c r="C151" s="2" t="s">
         <x:v>28</x:v>
       </x:c>
@@ -12670,7 +12692,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H151" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I151" s="56"/>
       <x:c r="J151" s="3"/>
@@ -12706,7 +12728,7 @@
         <x:v>572</x:v>
       </x:c>
       <x:c r="U151" s="2" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="152" ht="34.04999923706055" customHeight="1">
@@ -12730,7 +12752,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H152" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I152" s="55"/>
       <x:c r="J152" s="7"/>
@@ -12758,7 +12780,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U152" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="153" ht="34.04999923706055" customHeight="1">
@@ -12782,7 +12804,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H153" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I153" s="56"/>
       <x:c r="J153" s="3"/>
@@ -12810,7 +12832,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U153" s="2" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="154" ht="34.04999923706055" customHeight="1">
@@ -12834,7 +12856,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H154" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I154" s="55"/>
       <x:c r="J154" s="7"/>
@@ -12862,7 +12884,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U154" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="155" ht="34.04999923706055" customHeight="1">
@@ -12886,7 +12908,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H155" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I155" s="56"/>
       <x:c r="J155" s="3"/>
@@ -12914,7 +12936,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U155" s="2" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="156" ht="34.04999923706055" customHeight="1">
@@ -12938,7 +12960,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H156" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I156" s="55"/>
       <x:c r="J156" s="7"/>
@@ -12966,7 +12988,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U156" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="157" ht="34.04999923706055" customHeight="1">
@@ -12990,7 +13012,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H157" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I157" s="56"/>
       <x:c r="J157" s="3"/>
@@ -13018,7 +13040,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U157" s="2" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="158" ht="34.04999923706055" customHeight="1">
@@ -13042,7 +13064,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H158" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I158" s="55"/>
       <x:c r="J158" s="7"/>
@@ -13070,7 +13092,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U158" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="159" ht="34.04999923706055" customHeight="1">
@@ -13094,7 +13116,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H159" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I159" s="56"/>
       <x:c r="J159" s="3"/>
@@ -13122,7 +13144,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U159" s="2" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="160" ht="34.04999923706055" customHeight="1">
@@ -13146,7 +13168,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H160" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I160" s="55"/>
       <x:c r="J160" s="7"/>
@@ -13174,14 +13196,14 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U160" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="34.04999923706055" customHeight="1">
       <x:c r="A161" s="3">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="B161" s="3">
+      <x:c r="B161" s="3" t="n">
         <x:v>142</x:v>
       </x:c>
       <x:c r="C161" s="2" t="s">
@@ -13199,8 +13221,8 @@
       <x:c r="G161" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H161" s="3" t="s">
-        <x:v>27</x:v>
+      <x:c r="H161" s="3" t="str">
+        <x:v>Day 07</x:v>
       </x:c>
       <x:c r="I161" s="56">
         <x:v>46202</x:v>
@@ -13265,7 +13287,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H162" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I162" s="55"/>
       <x:c r="J162" s="7"/>
@@ -13293,7 +13315,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U162" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="163" ht="34.04999923706055" customHeight="1">
@@ -13317,7 +13339,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H163" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I163" s="56"/>
       <x:c r="J163" s="3"/>
@@ -13345,7 +13367,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U163" s="2" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="34.04999923706055" customHeight="1">
@@ -13576,7 +13598,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H167" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I167" s="56"/>
       <x:c r="J167" s="3"/>
@@ -13604,7 +13626,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U167" s="2" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="168" ht="34.04999923706055" customHeight="1">
@@ -13697,7 +13719,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H169" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I169" s="56"/>
       <x:c r="J169" s="3"/>
@@ -13725,7 +13747,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U169" s="2" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="170" ht="34.04999923706055" customHeight="1">
@@ -13749,7 +13771,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H170" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I170" s="55"/>
       <x:c r="J170" s="7"/>
@@ -13777,7 +13799,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U170" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="171" ht="34.04999923706055" customHeight="1">
@@ -13801,7 +13823,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H171" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I171" s="56"/>
       <x:c r="J171" s="3"/>
@@ -13829,7 +13851,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U171" s="2" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="172" ht="34.04999923706055" customHeight="1">
@@ -13853,7 +13875,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H172" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I172" s="55"/>
       <x:c r="J172" s="7"/>
@@ -13889,14 +13911,14 @@
         <x:v>616</x:v>
       </x:c>
       <x:c r="U172" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="173" ht="34.04999923706055" customHeight="1">
       <x:c r="A173" s="3">
         <x:v>151</x:v>
       </x:c>
-      <x:c r="B173" s="3">
+      <x:c r="B173" s="3" t="n">
         <x:v>121</x:v>
       </x:c>
       <x:c r="C173" s="2" t="s">
@@ -13914,8 +13936,8 @@
       <x:c r="G173" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H173" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H173" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I173" s="56">
         <x:v>46201</x:v>
@@ -13988,7 +14010,7 @@
       <x:c r="A175" s="7">
         <x:v>152</x:v>
       </x:c>
-      <x:c r="B175" s="7">
+      <x:c r="B175" s="7" t="n">
         <x:v>147</x:v>
       </x:c>
       <x:c r="C175" s="8" t="s">
@@ -14006,8 +14028,8 @@
       <x:c r="G175" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H175" s="7" t="s">
-        <x:v>32</x:v>
+      <x:c r="H175" s="7" t="str">
+        <x:v>Day 09</x:v>
       </x:c>
       <x:c r="I175" s="55">
         <x:v>46205</x:v>
@@ -14055,7 +14077,7 @@
       <x:c r="A176" s="3">
         <x:v>153</x:v>
       </x:c>
-      <x:c r="B176" s="3">
+      <x:c r="B176" s="3" t="n">
         <x:v>148</x:v>
       </x:c>
       <x:c r="C176" s="2" t="s">
@@ -14073,8 +14095,8 @@
       <x:c r="G176" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H176" s="3" t="s">
-        <x:v>32</x:v>
+      <x:c r="H176" s="3" t="str">
+        <x:v>Day 09</x:v>
       </x:c>
       <x:c r="I176" s="56">
         <x:v>46205</x:v>
@@ -14122,7 +14144,7 @@
       <x:c r="A177" s="7">
         <x:v>154</x:v>
       </x:c>
-      <x:c r="B177" s="7">
+      <x:c r="B177" s="7" t="n">
         <x:v>149</x:v>
       </x:c>
       <x:c r="C177" s="8" t="s">
@@ -14140,8 +14162,8 @@
       <x:c r="G177" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H177" s="7" t="s">
-        <x:v>32</x:v>
+      <x:c r="H177" s="7" t="str">
+        <x:v>Day 09</x:v>
       </x:c>
       <x:c r="I177" s="55">
         <x:v>46205</x:v>
@@ -14189,7 +14211,7 @@
       <x:c r="A178" s="3">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="B178" s="3">
+      <x:c r="B178" s="3" t="n">
         <x:v>150</x:v>
       </x:c>
       <x:c r="C178" s="2" t="s">
@@ -14207,8 +14229,8 @@
       <x:c r="G178" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H178" s="3" t="s">
-        <x:v>32</x:v>
+      <x:c r="H178" s="3" t="str">
+        <x:v>Day 09</x:v>
       </x:c>
       <x:c r="I178" s="56">
         <x:v>46205</x:v>
@@ -14407,7 +14429,7 @@
         <x:v>523</x:v>
       </x:c>
       <x:c r="H181" s="57" t="str">
-        <x:v>Day 11</x:v>
+        <x:v>Day 12</x:v>
       </x:c>
       <x:c r="I181" s="55"/>
       <x:c r="J181" s="7"/>
@@ -14435,7 +14457,7 @@
         <x:v>524</x:v>
       </x:c>
       <x:c r="U181" s="8" t="str">
-        <x:v>Planned for 2026-07-04. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
+        <x:v>Planned for 2026-07-05. Add the screenshot, solution, archive number, and actual submission timestamp only after HDLBits reports Success.</x:v>
       </x:c>
     </x:row>
     <x:row r="182" ht="25.049999237060547" customHeight="1">
@@ -14492,7 +14514,7 @@
       <x:c r="A184" s="3">
         <x:v>159</x:v>
       </x:c>
-      <x:c r="B184" s="3">
+      <x:c r="B184" s="3" t="n">
         <x:v>122</x:v>
       </x:c>
       <x:c r="C184" s="2" t="s">
@@ -14510,8 +14532,8 @@
       <x:c r="G184" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H184" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H184" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I184" s="56">
         <x:v>46201</x:v>
@@ -14559,7 +14581,7 @@
       <x:c r="A185" s="7">
         <x:v>160</x:v>
       </x:c>
-      <x:c r="B185" s="7">
+      <x:c r="B185" s="7" t="n">
         <x:v>123</x:v>
       </x:c>
       <x:c r="C185" s="8" t="s">
@@ -14577,8 +14599,8 @@
       <x:c r="G185" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H185" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="H185" s="7" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I185" s="55">
         <x:v>46201</x:v>
@@ -14626,7 +14648,7 @@
       <x:c r="A186" s="3">
         <x:v>161</x:v>
       </x:c>
-      <x:c r="B186" s="3">
+      <x:c r="B186" s="3" t="n">
         <x:v>124</x:v>
       </x:c>
       <x:c r="C186" s="2" t="s">
@@ -14644,8 +14666,8 @@
       <x:c r="G186" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H186" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H186" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I186" s="56">
         <x:v>46201</x:v>
@@ -14693,7 +14715,7 @@
       <x:c r="A187" s="7">
         <x:v>162</x:v>
       </x:c>
-      <x:c r="B187" s="7">
+      <x:c r="B187" s="7" t="n">
         <x:v>125</x:v>
       </x:c>
       <x:c r="C187" s="8" t="s">
@@ -14711,8 +14733,8 @@
       <x:c r="G187" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H187" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="H187" s="7" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I187" s="55">
         <x:v>46201</x:v>
@@ -14760,7 +14782,7 @@
       <x:c r="A188" s="3">
         <x:v>163</x:v>
       </x:c>
-      <x:c r="B188" s="3">
+      <x:c r="B188" s="3" t="n">
         <x:v>126</x:v>
       </x:c>
       <x:c r="C188" s="2" t="s">
@@ -14778,8 +14800,8 @@
       <x:c r="G188" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H188" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H188" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I188" s="56">
         <x:v>46201</x:v>
@@ -14852,7 +14874,7 @@
       <x:c r="A190" s="7">
         <x:v>164</x:v>
       </x:c>
-      <x:c r="B190" s="7">
+      <x:c r="B190" s="7" t="n">
         <x:v>127</x:v>
       </x:c>
       <x:c r="C190" s="8" t="s">
@@ -14870,8 +14892,8 @@
       <x:c r="G190" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H190" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="H190" s="7" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I190" s="55">
         <x:v>46201</x:v>
@@ -14919,7 +14941,7 @@
       <x:c r="A191" s="3">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="B191" s="3">
+      <x:c r="B191" s="3" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="C191" s="2" t="s">
@@ -14937,8 +14959,8 @@
       <x:c r="G191" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H191" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H191" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I191" s="56">
         <x:v>46201</x:v>
@@ -14986,7 +15008,7 @@
       <x:c r="A192" s="7">
         <x:v>166</x:v>
       </x:c>
-      <x:c r="B192" s="7">
+      <x:c r="B192" s="7" t="n">
         <x:v>129</x:v>
       </x:c>
       <x:c r="C192" s="8" t="s">
@@ -15004,8 +15026,8 @@
       <x:c r="G192" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H192" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="H192" s="7" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I192" s="55">
         <x:v>46201</x:v>
@@ -15053,7 +15075,7 @@
       <x:c r="A193" s="3">
         <x:v>167</x:v>
       </x:c>
-      <x:c r="B193" s="3">
+      <x:c r="B193" s="3" t="n">
         <x:v>130</x:v>
       </x:c>
       <x:c r="C193" s="2" t="s">
@@ -15071,8 +15093,8 @@
       <x:c r="G193" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H193" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H193" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I193" s="56">
         <x:v>46201</x:v>
@@ -15120,7 +15142,7 @@
       <x:c r="A194" s="7">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="B194" s="7">
+      <x:c r="B194" s="7" t="n">
         <x:v>131</x:v>
       </x:c>
       <x:c r="C194" s="8" t="s">
@@ -15138,8 +15160,8 @@
       <x:c r="G194" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H194" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="H194" s="7" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I194" s="55">
         <x:v>46201</x:v>
@@ -15187,7 +15209,7 @@
       <x:c r="A195" s="3">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="B195" s="3">
+      <x:c r="B195" s="3" t="n">
         <x:v>132</x:v>
       </x:c>
       <x:c r="C195" s="2" t="s">
@@ -15205,8 +15227,8 @@
       <x:c r="G195" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H195" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H195" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I195" s="56">
         <x:v>46201</x:v>
@@ -15254,7 +15276,7 @@
       <x:c r="A196" s="7">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="B196" s="7">
+      <x:c r="B196" s="7" t="n">
         <x:v>133</x:v>
       </x:c>
       <x:c r="C196" s="8" t="s">
@@ -15272,8 +15294,8 @@
       <x:c r="G196" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H196" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="H196" s="7" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I196" s="55">
         <x:v>46201</x:v>
@@ -15321,7 +15343,7 @@
       <x:c r="A197" s="3">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="B197" s="3">
+      <x:c r="B197" s="3" t="n">
         <x:v>134</x:v>
       </x:c>
       <x:c r="C197" s="2" t="s">
@@ -15339,8 +15361,8 @@
       <x:c r="G197" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H197" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H197" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I197" s="56">
         <x:v>46201</x:v>
@@ -15388,7 +15410,7 @@
       <x:c r="A198" s="7">
         <x:v>172</x:v>
       </x:c>
-      <x:c r="B198" s="7">
+      <x:c r="B198" s="7" t="n">
         <x:v>135</x:v>
       </x:c>
       <x:c r="C198" s="8" t="s">
@@ -15406,8 +15428,8 @@
       <x:c r="G198" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H198" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="H198" s="7" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I198" s="55">
         <x:v>46201</x:v>
@@ -15455,7 +15477,7 @@
       <x:c r="A199" s="3">
         <x:v>173</x:v>
       </x:c>
-      <x:c r="B199" s="3">
+      <x:c r="B199" s="3" t="n">
         <x:v>136</x:v>
       </x:c>
       <x:c r="C199" s="2" t="s">
@@ -15473,8 +15495,8 @@
       <x:c r="G199" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H199" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H199" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I199" s="56">
         <x:v>46201</x:v>
@@ -15547,7 +15569,7 @@
       <x:c r="A201" s="7">
         <x:v>174</x:v>
       </x:c>
-      <x:c r="B201" s="7">
+      <x:c r="B201" s="7" t="n">
         <x:v>137</x:v>
       </x:c>
       <x:c r="C201" s="8" t="s">
@@ -15563,8 +15585,8 @@
       <x:c r="G201" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H201" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="H201" s="7" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I201" s="55">
         <x:v>46201</x:v>
@@ -15612,7 +15634,7 @@
       <x:c r="A202" s="3">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="B202" s="3">
+      <x:c r="B202" s="3" t="n">
         <x:v>138</x:v>
       </x:c>
       <x:c r="C202" s="2" t="s">
@@ -15628,8 +15650,8 @@
       <x:c r="G202" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H202" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H202" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I202" s="56">
         <x:v>46201</x:v>
@@ -15677,7 +15699,7 @@
       <x:c r="A203" s="7">
         <x:v>176</x:v>
       </x:c>
-      <x:c r="B203" s="7">
+      <x:c r="B203" s="7" t="n">
         <x:v>139</x:v>
       </x:c>
       <x:c r="C203" s="8" t="s">
@@ -15693,8 +15715,8 @@
       <x:c r="G203" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H203" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="H203" s="7" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I203" s="55">
         <x:v>46201</x:v>
@@ -15742,7 +15764,7 @@
       <x:c r="A204" s="3">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="B204" s="3">
+      <x:c r="B204" s="3" t="n">
         <x:v>140</x:v>
       </x:c>
       <x:c r="C204" s="2" t="s">
@@ -15758,8 +15780,8 @@
       <x:c r="G204" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H204" s="3" t="s">
-        <x:v>25</x:v>
+      <x:c r="H204" s="3" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I204" s="56">
         <x:v>46201</x:v>
@@ -15807,7 +15829,7 @@
       <x:c r="A205" s="12">
         <x:v>178</x:v>
       </x:c>
-      <x:c r="B205" s="12">
+      <x:c r="B205" s="12" t="n">
         <x:v>141</x:v>
       </x:c>
       <x:c r="C205" s="13" t="s">
@@ -15823,8 +15845,8 @@
       <x:c r="G205" s="12" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H205" s="12" t="s">
-        <x:v>25</x:v>
+      <x:c r="H205" s="12" t="str">
+        <x:v>Day 06</x:v>
       </x:c>
       <x:c r="I205" s="61">
         <x:v>46201</x:v>

</xml_diff>